<commit_message>
Use hot cup and lid for hot coffee recipes
Co-authored-by: jjimenezdev23 <jjimenezdev23@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/coffee_capital_system.xlsx
+++ b/coffee_capital_system.xlsx
@@ -215,8 +215,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnitCosts" displayName="UnitCosts" ref="A1:F12" headerRowCount="1">
-  <autoFilter ref="A1:F12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnitCosts" displayName="UnitCosts" ref="A1:F14" headerRowCount="1">
+  <autoFilter ref="A1:F14"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Ingredient"/>
     <tableColumn id="2" name="Measurement Unit"/>
@@ -230,9 +230,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecipeUsage" displayName="RecipeUsage" ref="A1:N14" headerRowCount="1">
-  <autoFilter ref="A1:N14"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RecipeUsage" displayName="RecipeUsage" ref="A1:P14" headerRowCount="1">
+  <autoFilter ref="A1:P14"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="Type"/>
     <tableColumn id="2" name="Recipe"/>
     <tableColumn id="3" name="Selling Price"/>
@@ -246,7 +246,9 @@
     <tableColumn id="11" name="Chocolate Syrup (g)"/>
     <tableColumn id="12" name="Cup (pc)"/>
     <tableColumn id="13" name="Lid (pc)"/>
-    <tableColumn id="14" name="Straw (pc)"/>
+    <tableColumn id="14" name="Hot Cup (pc)"/>
+    <tableColumn id="15" name="Hot Lid (pc)"/>
+    <tableColumn id="16" name="Straw (pc)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -678,7 +680,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Hot coffee base data mentioned Straw, but hot recipes did not list Straw; hot recipe straw quantity is set to 0. Change Recipe Usage if you include a straw or stirrer.</t>
+          <t>Iced recipes use the Cup and Lid cost inputs; hot recipes use the separate Hot Cup and Hot Lid cost inputs.</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -686,7 +688,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Water cost can be entered as 0 if you do not track it separately.</t>
+          <t>Hot coffee base data mentioned Straw, but hot recipes did not list Straw; hot recipe straw quantity is set to 0. Change Recipe Usage if you include a straw or stirrer.</t>
         </is>
       </c>
       <c r="B15" s="2" t="n"/>
@@ -694,13 +696,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Water cost can be entered as 0 if you do not track it separately.</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>All costs should be entered in the same currency as your selling prices.</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
       <c r="B17" s="2" t="n"/>
     </row>
     <row r="18">
@@ -774,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -882,7 +888,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Enter number of cups per pack and pack cost.</t>
+          <t>Enter number of iced/cold cups per pack and pack cost.</t>
         </is>
       </c>
     </row>
@@ -905,19 +911,19 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Enter number of lids per pack and pack cost.</t>
+          <t>Enter number of iced/cold lids per pack and pack cost.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="C6" s="8" t="n"/>
@@ -928,14 +934,14 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Enter total grams bought/produced and cost.</t>
+          <t>Enter number of hot cups per pack and pack cost.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Straw</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -951,19 +957,19 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Enter number of straws per pack and pack cost.</t>
+          <t>Enter number of hot lids per pack and pack cost.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>g</t>
         </is>
       </c>
       <c r="C8" s="8" t="n"/>
@@ -974,19 +980,19 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Enter total ml and cost if you want to include water.</t>
+          <t>Enter total grams bought/produced and cost.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Condensed milk</t>
+          <t>Straw</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="C9" s="8" t="n"/>
@@ -997,19 +1003,19 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Enter can/container total grams and cost.</t>
+          <t>Enter number of straws per pack and pack cost.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ube powder</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>ml</t>
         </is>
       </c>
       <c r="C10" s="8" t="n"/>
@@ -1020,14 +1026,14 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Enter pouch/container total grams and cost.</t>
+          <t>Enter total ml and cost if you want to include water.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Caramel Syrup</t>
+          <t>Condensed milk</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1043,14 +1049,14 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Enter bottle total grams and cost.</t>
+          <t>Enter can/container total grams and cost.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Chocolate Syrup</t>
+          <t>Ube powder</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1065,6 +1071,52 @@
         <v/>
       </c>
       <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Enter pouch/container total grams and cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Caramel Syrup</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="9">
+        <f>IF(OR(C13="",D13=""),"",D13/C13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Enter bottle total grams and cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chocolate Syrup</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="9">
+        <f>IF(OR(C14="",D14=""),"",D14/C14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Enter bottle total grams and cost.</t>
         </is>
@@ -1084,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1100,7 +1152,9 @@
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1171,6 +1225,16 @@
       </c>
       <c r="N1" s="6" t="inlineStr">
         <is>
+          <t>Hot Cup (pc)</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Hot Lid (pc)</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
           <t>Straw (pc)</t>
         </is>
       </c>
@@ -1220,6 +1284,12 @@
         <v>1</v>
       </c>
       <c r="N2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1268,6 +1338,12 @@
         <v>1</v>
       </c>
       <c r="N3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1316,6 +1392,12 @@
         <v>1</v>
       </c>
       <c r="N4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1364,6 +1446,12 @@
         <v>1</v>
       </c>
       <c r="N5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1412,6 +1500,12 @@
         <v>1</v>
       </c>
       <c r="N6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1460,6 +1554,12 @@
         <v>1</v>
       </c>
       <c r="N7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1508,6 +1608,12 @@
         <v>1</v>
       </c>
       <c r="N8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1550,12 +1656,18 @@
         <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1598,12 +1710,18 @@
         <v>0</v>
       </c>
       <c r="L10" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1646,12 +1764,18 @@
         <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1694,12 +1818,18 @@
         <v>0</v>
       </c>
       <c r="L12" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1742,12 +1872,18 @@
         <v>35</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1790,12 +1926,18 @@
         <v>0</v>
       </c>
       <c r="L14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1896,7 +2038,7 @@
         </is>
       </c>
       <c r="G2" s="9">
-        <f>IFERROR(VLOOKUP(D2,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D2,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H2" s="11">
@@ -1932,7 +2074,7 @@
         </is>
       </c>
       <c r="G3" s="9">
-        <f>IFERROR(VLOOKUP(D3,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D3,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H3" s="11">
@@ -1968,7 +2110,7 @@
         </is>
       </c>
       <c r="G4" s="9">
-        <f>IFERROR(VLOOKUP(D4,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D4,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H4" s="11">
@@ -2004,7 +2146,7 @@
         </is>
       </c>
       <c r="G5" s="9">
-        <f>IFERROR(VLOOKUP(D5,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D5,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H5" s="11">
@@ -2040,7 +2182,7 @@
         </is>
       </c>
       <c r="G6" s="9">
-        <f>IFERROR(VLOOKUP(D6,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D6,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H6" s="11">
@@ -2076,7 +2218,7 @@
         </is>
       </c>
       <c r="G7" s="9">
-        <f>IFERROR(VLOOKUP(D7,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D7,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H7" s="11">
@@ -2112,7 +2254,7 @@
         </is>
       </c>
       <c r="G8" s="9">
-        <f>IFERROR(VLOOKUP(D8,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D8,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H8" s="11">
@@ -2148,7 +2290,7 @@
         </is>
       </c>
       <c r="G9" s="9">
-        <f>IFERROR(VLOOKUP(D9,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D9,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H9" s="11">
@@ -2184,7 +2326,7 @@
         </is>
       </c>
       <c r="G10" s="9">
-        <f>IFERROR(VLOOKUP(D10,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D10,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H10" s="11">
@@ -2220,7 +2362,7 @@
         </is>
       </c>
       <c r="G11" s="9">
-        <f>IFERROR(VLOOKUP(D11,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D11,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H11" s="11">
@@ -2256,7 +2398,7 @@
         </is>
       </c>
       <c r="G12" s="9">
-        <f>IFERROR(VLOOKUP(D12,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D12,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H12" s="11">
@@ -2292,7 +2434,7 @@
         </is>
       </c>
       <c r="G13" s="9">
-        <f>IFERROR(VLOOKUP(D13,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D13,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H13" s="11">
@@ -2328,7 +2470,7 @@
         </is>
       </c>
       <c r="G14" s="9">
-        <f>IFERROR(VLOOKUP(D14,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D14,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H14" s="11">
@@ -2364,7 +2506,7 @@
         </is>
       </c>
       <c r="G15" s="9">
-        <f>IFERROR(VLOOKUP(D15,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D15,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H15" s="11">
@@ -2400,7 +2542,7 @@
         </is>
       </c>
       <c r="G16" s="9">
-        <f>IFERROR(VLOOKUP(D16,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D16,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H16" s="11">
@@ -2436,7 +2578,7 @@
         </is>
       </c>
       <c r="G17" s="9">
-        <f>IFERROR(VLOOKUP(D17,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D17,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H17" s="11">
@@ -2472,7 +2614,7 @@
         </is>
       </c>
       <c r="G18" s="9">
-        <f>IFERROR(VLOOKUP(D18,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D18,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H18" s="11">
@@ -2508,7 +2650,7 @@
         </is>
       </c>
       <c r="G19" s="9">
-        <f>IFERROR(VLOOKUP(D19,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D19,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H19" s="11">
@@ -2544,7 +2686,7 @@
         </is>
       </c>
       <c r="G20" s="9">
-        <f>IFERROR(VLOOKUP(D20,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D20,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H20" s="11">
@@ -2580,7 +2722,7 @@
         </is>
       </c>
       <c r="G21" s="9">
-        <f>IFERROR(VLOOKUP(D21,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D21,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H21" s="11">
@@ -2616,7 +2758,7 @@
         </is>
       </c>
       <c r="G22" s="9">
-        <f>IFERROR(VLOOKUP(D22,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D22,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H22" s="11">
@@ -2652,7 +2794,7 @@
         </is>
       </c>
       <c r="G23" s="9">
-        <f>IFERROR(VLOOKUP(D23,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D23,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H23" s="11">
@@ -2688,7 +2830,7 @@
         </is>
       </c>
       <c r="G24" s="9">
-        <f>IFERROR(VLOOKUP(D24,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D24,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H24" s="11">
@@ -2724,7 +2866,7 @@
         </is>
       </c>
       <c r="G25" s="9">
-        <f>IFERROR(VLOOKUP(D25,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D25,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H25" s="11">
@@ -2760,7 +2902,7 @@
         </is>
       </c>
       <c r="G26" s="9">
-        <f>IFERROR(VLOOKUP(D26,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D26,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H26" s="11">
@@ -2796,7 +2938,7 @@
         </is>
       </c>
       <c r="G27" s="9">
-        <f>IFERROR(VLOOKUP(D27,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D27,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H27" s="11">
@@ -2832,7 +2974,7 @@
         </is>
       </c>
       <c r="G28" s="9">
-        <f>IFERROR(VLOOKUP(D28,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D28,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H28" s="11">
@@ -2868,7 +3010,7 @@
         </is>
       </c>
       <c r="G29" s="9">
-        <f>IFERROR(VLOOKUP(D29,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D29,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H29" s="11">
@@ -2904,7 +3046,7 @@
         </is>
       </c>
       <c r="G30" s="9">
-        <f>IFERROR(VLOOKUP(D30,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D30,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H30" s="11">
@@ -2940,7 +3082,7 @@
         </is>
       </c>
       <c r="G31" s="9">
-        <f>IFERROR(VLOOKUP(D31,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D31,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H31" s="11">
@@ -2976,7 +3118,7 @@
         </is>
       </c>
       <c r="G32" s="9">
-        <f>IFERROR(VLOOKUP(D32,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D32,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H32" s="11">
@@ -3012,7 +3154,7 @@
         </is>
       </c>
       <c r="G33" s="9">
-        <f>IFERROR(VLOOKUP(D33,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D33,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H33" s="11">
@@ -3048,7 +3190,7 @@
         </is>
       </c>
       <c r="G34" s="9">
-        <f>IFERROR(VLOOKUP(D34,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D34,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H34" s="11">
@@ -3084,7 +3226,7 @@
         </is>
       </c>
       <c r="G35" s="9">
-        <f>IFERROR(VLOOKUP(D35,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D35,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H35" s="11">
@@ -3120,7 +3262,7 @@
         </is>
       </c>
       <c r="G36" s="9">
-        <f>IFERROR(VLOOKUP(D36,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D36,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H36" s="11">
@@ -3156,7 +3298,7 @@
         </is>
       </c>
       <c r="G37" s="9">
-        <f>IFERROR(VLOOKUP(D37,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D37,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H37" s="11">
@@ -3192,7 +3334,7 @@
         </is>
       </c>
       <c r="G38" s="9">
-        <f>IFERROR(VLOOKUP(D38,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D38,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H38" s="11">
@@ -3228,7 +3370,7 @@
         </is>
       </c>
       <c r="G39" s="9">
-        <f>IFERROR(VLOOKUP(D39,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D39,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H39" s="11">
@@ -3264,7 +3406,7 @@
         </is>
       </c>
       <c r="G40" s="9">
-        <f>IFERROR(VLOOKUP(D40,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D40,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H40" s="11">
@@ -3300,7 +3442,7 @@
         </is>
       </c>
       <c r="G41" s="9">
-        <f>IFERROR(VLOOKUP(D41,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D41,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H41" s="11">
@@ -3336,7 +3478,7 @@
         </is>
       </c>
       <c r="G42" s="9">
-        <f>IFERROR(VLOOKUP(D42,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D42,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H42" s="11">
@@ -3372,7 +3514,7 @@
         </is>
       </c>
       <c r="G43" s="9">
-        <f>IFERROR(VLOOKUP(D43,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D43,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H43" s="11">
@@ -3408,7 +3550,7 @@
         </is>
       </c>
       <c r="G44" s="9">
-        <f>IFERROR(VLOOKUP(D44,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D44,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H44" s="11">
@@ -3444,7 +3586,7 @@
         </is>
       </c>
       <c r="G45" s="9">
-        <f>IFERROR(VLOOKUP(D45,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D45,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H45" s="11">
@@ -3480,7 +3622,7 @@
         </is>
       </c>
       <c r="G46" s="9">
-        <f>IFERROR(VLOOKUP(D46,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D46,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H46" s="11">
@@ -3516,7 +3658,7 @@
         </is>
       </c>
       <c r="G47" s="9">
-        <f>IFERROR(VLOOKUP(D47,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D47,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H47" s="11">
@@ -3552,7 +3694,7 @@
         </is>
       </c>
       <c r="G48" s="9">
-        <f>IFERROR(VLOOKUP(D48,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D48,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H48" s="11">
@@ -3588,7 +3730,7 @@
         </is>
       </c>
       <c r="G49" s="9">
-        <f>IFERROR(VLOOKUP(D49,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D49,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H49" s="11">
@@ -3624,7 +3766,7 @@
         </is>
       </c>
       <c r="G50" s="9">
-        <f>IFERROR(VLOOKUP(D50,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D50,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H50" s="11">
@@ -3660,7 +3802,7 @@
         </is>
       </c>
       <c r="G51" s="9">
-        <f>IFERROR(VLOOKUP(D51,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D51,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H51" s="11">
@@ -3696,7 +3838,7 @@
         </is>
       </c>
       <c r="G52" s="9">
-        <f>IFERROR(VLOOKUP(D52,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D52,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H52" s="11">
@@ -3732,7 +3874,7 @@
         </is>
       </c>
       <c r="G53" s="9">
-        <f>IFERROR(VLOOKUP(D53,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D53,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H53" s="11">
@@ -3768,7 +3910,7 @@
         </is>
       </c>
       <c r="G54" s="9">
-        <f>IFERROR(VLOOKUP(D54,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D54,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H54" s="11">
@@ -3792,7 +3934,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E55" s="10" t="n">
@@ -3804,7 +3946,7 @@
         </is>
       </c>
       <c r="G55" s="9">
-        <f>IFERROR(VLOOKUP(D55,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D55,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H55" s="11">
@@ -3828,7 +3970,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E56" s="10" t="n">
@@ -3840,7 +3982,7 @@
         </is>
       </c>
       <c r="G56" s="9">
-        <f>IFERROR(VLOOKUP(D56,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D56,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H56" s="11">
@@ -3876,7 +4018,7 @@
         </is>
       </c>
       <c r="G57" s="9">
-        <f>IFERROR(VLOOKUP(D57,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D57,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H57" s="11">
@@ -3912,7 +4054,7 @@
         </is>
       </c>
       <c r="G58" s="9">
-        <f>IFERROR(VLOOKUP(D58,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D58,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H58" s="11">
@@ -3936,7 +4078,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E59" s="10" t="n">
@@ -3948,7 +4090,7 @@
         </is>
       </c>
       <c r="G59" s="9">
-        <f>IFERROR(VLOOKUP(D59,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D59,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H59" s="11">
@@ -3972,7 +4114,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E60" s="10" t="n">
@@ -3984,7 +4126,7 @@
         </is>
       </c>
       <c r="G60" s="9">
-        <f>IFERROR(VLOOKUP(D60,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D60,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H60" s="11">
@@ -4020,7 +4162,7 @@
         </is>
       </c>
       <c r="G61" s="9">
-        <f>IFERROR(VLOOKUP(D61,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D61,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H61" s="11">
@@ -4056,7 +4198,7 @@
         </is>
       </c>
       <c r="G62" s="9">
-        <f>IFERROR(VLOOKUP(D62,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D62,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H62" s="11">
@@ -4080,7 +4222,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E63" s="10" t="n">
@@ -4092,7 +4234,7 @@
         </is>
       </c>
       <c r="G63" s="9">
-        <f>IFERROR(VLOOKUP(D63,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D63,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H63" s="11">
@@ -4116,7 +4258,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E64" s="10" t="n">
@@ -4128,7 +4270,7 @@
         </is>
       </c>
       <c r="G64" s="9">
-        <f>IFERROR(VLOOKUP(D64,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D64,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H64" s="11">
@@ -4164,7 +4306,7 @@
         </is>
       </c>
       <c r="G65" s="9">
-        <f>IFERROR(VLOOKUP(D65,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D65,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H65" s="11">
@@ -4200,7 +4342,7 @@
         </is>
       </c>
       <c r="G66" s="9">
-        <f>IFERROR(VLOOKUP(D66,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D66,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H66" s="11">
@@ -4236,7 +4378,7 @@
         </is>
       </c>
       <c r="G67" s="9">
-        <f>IFERROR(VLOOKUP(D67,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D67,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H67" s="11">
@@ -4272,7 +4414,7 @@
         </is>
       </c>
       <c r="G68" s="9">
-        <f>IFERROR(VLOOKUP(D68,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D68,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H68" s="11">
@@ -4296,7 +4438,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E69" s="10" t="n">
@@ -4308,7 +4450,7 @@
         </is>
       </c>
       <c r="G69" s="9">
-        <f>IFERROR(VLOOKUP(D69,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D69,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H69" s="11">
@@ -4332,7 +4474,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E70" s="10" t="n">
@@ -4344,7 +4486,7 @@
         </is>
       </c>
       <c r="G70" s="9">
-        <f>IFERROR(VLOOKUP(D70,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D70,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H70" s="11">
@@ -4380,7 +4522,7 @@
         </is>
       </c>
       <c r="G71" s="9">
-        <f>IFERROR(VLOOKUP(D71,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D71,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H71" s="11">
@@ -4416,7 +4558,7 @@
         </is>
       </c>
       <c r="G72" s="9">
-        <f>IFERROR(VLOOKUP(D72,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D72,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H72" s="11">
@@ -4452,7 +4594,7 @@
         </is>
       </c>
       <c r="G73" s="9">
-        <f>IFERROR(VLOOKUP(D73,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D73,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H73" s="11">
@@ -4488,7 +4630,7 @@
         </is>
       </c>
       <c r="G74" s="9">
-        <f>IFERROR(VLOOKUP(D74,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D74,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H74" s="11">
@@ -4512,7 +4654,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E75" s="10" t="n">
@@ -4524,7 +4666,7 @@
         </is>
       </c>
       <c r="G75" s="9">
-        <f>IFERROR(VLOOKUP(D75,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D75,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H75" s="11">
@@ -4548,7 +4690,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E76" s="10" t="n">
@@ -4560,7 +4702,7 @@
         </is>
       </c>
       <c r="G76" s="9">
-        <f>IFERROR(VLOOKUP(D76,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D76,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H76" s="11">
@@ -4596,7 +4738,7 @@
         </is>
       </c>
       <c r="G77" s="9">
-        <f>IFERROR(VLOOKUP(D77,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D77,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H77" s="11">
@@ -4632,7 +4774,7 @@
         </is>
       </c>
       <c r="G78" s="9">
-        <f>IFERROR(VLOOKUP(D78,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D78,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H78" s="11">
@@ -4668,7 +4810,7 @@
         </is>
       </c>
       <c r="G79" s="9">
-        <f>IFERROR(VLOOKUP(D79,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D79,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H79" s="11">
@@ -4704,7 +4846,7 @@
         </is>
       </c>
       <c r="G80" s="9">
-        <f>IFERROR(VLOOKUP(D80,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D80,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H80" s="11">
@@ -4728,7 +4870,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Cup</t>
+          <t>Hot Cup</t>
         </is>
       </c>
       <c r="E81" s="10" t="n">
@@ -4740,7 +4882,7 @@
         </is>
       </c>
       <c r="G81" s="9">
-        <f>IFERROR(VLOOKUP(D81,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D81,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H81" s="11">
@@ -4764,7 +4906,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Lid</t>
+          <t>Hot Lid</t>
         </is>
       </c>
       <c r="E82" s="10" t="n">
@@ -4776,7 +4918,7 @@
         </is>
       </c>
       <c r="G82" s="9">
-        <f>IFERROR(VLOOKUP(D82,'Unit Costs'!$A$2:$E$12,5,FALSE),"")</f>
+        <f>IFERROR(VLOOKUP(D82,'Unit Costs'!$A$2:$E$14,5,FALSE),"")</f>
         <v/>
       </c>
       <c r="H82" s="11">

</xml_diff>